<commit_message>
Correct Switchboard MMS rate to $0.030 per campaign-confirmed pricing
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UFnECcgtAfYRHFtdTfRTQd
</commit_message>
<xml_diff>
--- a/acquisition-estimator.xlsx
+++ b/acquisition-estimator.xlsx
@@ -264,10 +264,10 @@
     <t xml:space="preserve">MMS (media attached / long message)</t>
   </si>
   <si>
-    <t xml:space="preserve">Flat rate - cheaper than a 2-segment SMS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Source: Switchboard published pricing (welcome.oneswitchboard.com/pricing and oneswitchboard.helpdocs.io 'Texting Pricing'), accessed 2026-07-23. Rates for registered/verified 10DLC traffic, inclusive of telecom fees, same for local or toll-free numbers. No monthly fee, no setup fee, no minimums or prepayment; inbound replies, landline cleaning, and errored messages are free; new accounts get a $30 trial credit. Blue cells are editable if Switchboard's rates change - the Estimator pulls from this table. Follow-up conversation messages are costed at the SMS 1-segment rate (cell B3).</t>
+    <t xml:space="preserve">Flat rate - same as a 2-segment SMS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rates confirmed by campaign, 2026-07-23: $0.015 per SMS segment, $0.030 per MMS (pay-as-you-go; see welcome.oneswitchboard.com/pricing). No monthly fee, no setup fee, no minimums or prepayment; inbound replies, landline cleaning, and errored messages are free. Blue cells are editable if rates change - the Estimator pulls from this table. Follow-up conversation messages are costed at the SMS 1-segment rate (cell B3).</t>
   </si>
   <si>
     <t xml:space="preserve">Budget Scenarios - Minimum vs. High</t>
@@ -461,32 +461,36 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -494,79 +498,79 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="172" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="173" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -594,27 +598,27 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="172" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -889,535 +893,535 @@
   <dimension ref="A1:D51"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="37"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="58"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+      <c r="B5" s="5"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="6" t="n">
+      <c r="B6" s="7" t="n">
         <v>10000</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="8" t="n">
+      <c r="B7" s="9" t="n">
         <v>1.5</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="8" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="9" t="n">
+      <c r="B8" s="10" t="n">
         <v>100000</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="8" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="s">
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="8" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="12" t="n">
         <f aca="false">INDEX('Switchboard Rates'!$B$3:$B$6,MATCH($B$11,'Switchboard Rates'!$A$3:$A$6,0))</f>
         <v>0.03</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="8" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="11" t="n">
+      <c r="B13" s="12" t="n">
         <f aca="false">'Switchboard Rates'!$B$3</f>
         <v>0.015</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="8" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B14" s="9" t="n">
+      <c r="B14" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="12" t="n">
+      <c r="B15" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="8" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B17" s="4"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="13" t="s">
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B18" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="C18" s="13" t="s">
+      <c r="C18" s="14" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="14" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="B19" s="15" t="n">
+      <c r="B19" s="16" t="n">
         <v>0.93</v>
       </c>
-      <c r="C19" s="15" t="n">
+      <c r="C19" s="16" t="n">
         <v>0.97</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="D19" s="8" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="14" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="B20" s="15" t="n">
+      <c r="B20" s="16" t="n">
         <v>0.04</v>
       </c>
-      <c r="C20" s="15" t="n">
+      <c r="C20" s="16" t="n">
         <v>0.12</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="D20" s="8" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="14" t="s">
+    <row r="21" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="B21" s="16" t="n">
+      <c r="B21" s="17" t="n">
         <v>0.001</v>
       </c>
-      <c r="C21" s="16" t="n">
+      <c r="C21" s="17" t="n">
         <v>0.005</v>
       </c>
-      <c r="D21" s="7" t="s">
+      <c r="D21" s="8" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="14" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="B22" s="6" t="n">
+      <c r="B22" s="7" t="n">
         <v>25</v>
       </c>
-      <c r="C22" s="6" t="n">
+      <c r="C22" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="D22" s="8" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="14" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="B23" s="17" t="n">
+      <c r="B23" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="C23" s="17" t="n">
+      <c r="C23" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="D23" s="8" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="14" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="B24" s="6" t="n">
+      <c r="B24" s="7" t="n">
         <v>25</v>
       </c>
-      <c r="C24" s="6" t="n">
+      <c r="C24" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="D24" s="7" t="s">
+      <c r="D24" s="8" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="3" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B26" s="4"/>
-      <c r="C26" s="4"/>
-      <c r="D26" s="4"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="13" t="s">
+      <c r="B26" s="5"/>
+      <c r="C26" s="5"/>
+      <c r="D26" s="5"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B27" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="C27" s="13" t="s">
+      <c r="C27" s="14" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="14" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="B28" s="18" t="n">
+      <c r="B28" s="19" t="n">
         <f aca="false">$B$12+B19*B20*$B$14*$B$13+$B$15</f>
         <v>0.031674</v>
       </c>
-      <c r="C28" s="18" t="n">
+      <c r="C28" s="19" t="n">
         <f aca="false">$B$12+C19*C20*$B$14*$B$13+$B$15</f>
         <v>0.035238</v>
       </c>
-      <c r="D28" s="7" t="s">
+      <c r="D28" s="8" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="14" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="B29" s="19" t="n">
+      <c r="B29" s="20" t="n">
         <f aca="false">IF(B28&gt;0,MIN($B$8,ROUNDDOWN($B$6/B28,0)),0)</f>
         <v>100000</v>
       </c>
-      <c r="C29" s="19" t="n">
+      <c r="C29" s="20" t="n">
         <f aca="false">IF(C28&gt;0,MIN($B$8,ROUNDDOWN($B$6/C28,0)),0)</f>
         <v>100000</v>
       </c>
-      <c r="D29" s="7" t="s">
+      <c r="D29" s="8" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="14" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="B30" s="20" t="n">
+      <c r="B30" s="21" t="n">
         <f aca="false">B29*B28</f>
         <v>3167.4</v>
       </c>
-      <c r="C30" s="20" t="n">
+      <c r="C30" s="21" t="n">
         <f aca="false">C29*C28</f>
         <v>3523.8</v>
       </c>
-      <c r="D30" s="7" t="s">
+      <c r="D30" s="8" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="14" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="B31" s="20" t="n">
+      <c r="B31" s="21" t="n">
         <f aca="false">$B$6-B30</f>
         <v>6832.6</v>
       </c>
-      <c r="C31" s="20" t="n">
+      <c r="C31" s="21" t="n">
         <f aca="false">$B$6-C30</f>
         <v>6476.2</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="14" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="B32" s="19" t="n">
+      <c r="B32" s="20" t="n">
         <f aca="false">B29*B19</f>
         <v>93000</v>
       </c>
-      <c r="C32" s="19" t="n">
+      <c r="C32" s="20" t="n">
         <f aca="false">C29*C19</f>
         <v>97000</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="14" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="B33" s="19" t="n">
+      <c r="B33" s="20" t="n">
         <f aca="false">B32*B20</f>
         <v>3720</v>
       </c>
-      <c r="C33" s="19" t="n">
+      <c r="C33" s="20" t="n">
         <f aca="false">C32*C20</f>
         <v>11640</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="5" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="B34" s="21" t="n">
+      <c r="B34" s="22" t="n">
         <f aca="false">B32*B21</f>
         <v>93</v>
       </c>
-      <c r="C34" s="21" t="n">
+      <c r="C34" s="22" t="n">
         <f aca="false">C32*C21</f>
         <v>485</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="5" t="s">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="B35" s="22" t="n">
+      <c r="B35" s="23" t="n">
         <f aca="false">IF(B34&gt;0,B30/B34,"n/a")</f>
         <v>34.058064516129</v>
       </c>
-      <c r="C35" s="22" t="n">
+      <c r="C35" s="23" t="n">
         <f aca="false">IF(C34&gt;0,C30/C34,"n/a")</f>
         <v>7.26556701030928</v>
       </c>
-      <c r="D35" s="7" t="s">
+      <c r="D35" s="8" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="14" t="s">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="B36" s="20" t="n">
+      <c r="B36" s="21" t="n">
         <f aca="false">B34*B22</f>
         <v>2325</v>
       </c>
-      <c r="C36" s="20" t="n">
+      <c r="C36" s="21" t="n">
         <f aca="false">C34*C22</f>
         <v>16975</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="14" t="s">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="B37" s="20" t="n">
+      <c r="B37" s="21" t="n">
         <f aca="false">B34*(B22+B23*B24)</f>
         <v>4650</v>
       </c>
-      <c r="C37" s="20" t="n">
+      <c r="C37" s="21" t="n">
         <f aca="false">C34*(C22+C23*C24)</f>
         <v>50925</v>
       </c>
-      <c r="D37" s="7" t="s">
+      <c r="D37" s="8" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="5" t="s">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="B38" s="23" t="n">
+      <c r="B38" s="24" t="n">
         <f aca="false">IF(B30&gt;0,(B37-B30)/B30,0)</f>
         <v>0.468081075961356</v>
       </c>
-      <c r="C38" s="23" t="n">
+      <c r="C38" s="24" t="n">
         <f aca="false">IF(C30&gt;0,(C37-C30)/C30,0)</f>
         <v>13.4517282479142</v>
       </c>
-      <c r="D38" s="7" t="s">
+      <c r="D38" s="8" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="14" t="s">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="B39" s="24" t="n">
+      <c r="B39" s="25" t="n">
         <f aca="false">IF(B30&gt;0,B37/B30,0)</f>
         <v>1.46808107596136</v>
       </c>
-      <c r="C39" s="24" t="n">
+      <c r="C39" s="25" t="n">
         <f aca="false">IF(C30&gt;0,C37/C30,0)</f>
         <v>14.4517282479142</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="5" t="s">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B40" s="25" t="str">
+      <c r="B40" s="26" t="str">
         <f aca="false">IF(B38&gt;=$B$7,"MEETS TARGET","BELOW TARGET")</f>
         <v>BELOW TARGET</v>
       </c>
-      <c r="C40" s="25" t="str">
+      <c r="C40" s="26" t="str">
         <f aca="false">IF(C38&gt;=$B$7,"MEETS TARGET","BELOW TARGET")</f>
         <v>MEETS TARGET</v>
       </c>
-      <c r="D40" s="7" t="s">
+      <c r="D40" s="8" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="3" t="s">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B42" s="4"/>
-      <c r="C42" s="4"/>
-      <c r="D42" s="4"/>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="14" t="s">
+      <c r="B42" s="5"/>
+      <c r="C42" s="5"/>
+      <c r="D42" s="5"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="15" t="s">
         <v>61</v>
       </c>
-      <c r="B43" s="20" t="n">
+      <c r="B43" s="21" t="n">
         <f aca="false">B22+B23*B24</f>
         <v>50</v>
       </c>
-      <c r="C43" s="20" t="n">
+      <c r="C43" s="21" t="n">
         <f aca="false">C22+C23*C24</f>
         <v>105</v>
       </c>
-      <c r="D43" s="7" t="s">
+      <c r="D43" s="8" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="5" t="s">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="B44" s="22" t="n">
+      <c r="B44" s="23" t="n">
         <f aca="false">B43/(1+$B$7)</f>
         <v>20</v>
       </c>
-      <c r="C44" s="22" t="n">
+      <c r="C44" s="23" t="n">
         <f aca="false">C43/(1+$B$7)</f>
         <v>42</v>
       </c>
-      <c r="D44" s="7" t="s">
+      <c r="D44" s="8" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="14" t="s">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="B45" s="19" t="n">
+      <c r="B45" s="20" t="n">
         <f aca="false">IF(B43&gt;0,(1+$B$7)*B30/B43,0)</f>
         <v>158.37</v>
       </c>
-      <c r="C45" s="19" t="n">
+      <c r="C45" s="20" t="n">
         <f aca="false">IF(C43&gt;0,(1+$B$7)*C30/C43,0)</f>
         <v>83.9</v>
       </c>
-      <c r="D45" s="7" t="s">
+      <c r="D45" s="8" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="14" t="s">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="15" t="s">
         <v>67</v>
       </c>
-      <c r="B46" s="26" t="n">
+      <c r="B46" s="27" t="n">
         <f aca="false">IF(B32&gt;0,B45/B32,0)</f>
         <v>0.00170290322580645</v>
       </c>
-      <c r="C46" s="26" t="n">
+      <c r="C46" s="27" t="n">
         <f aca="false">IF(C32&gt;0,C45/C32,0)</f>
         <v>0.000864948453608248</v>
       </c>
-      <c r="D46" s="7" t="s">
+      <c r="D46" s="8" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="27" t="s">
+      <c r="A48" s="28" t="s">
         <v>69</v>
       </c>
-      <c r="B48" s="27"/>
-      <c r="C48" s="27"/>
-      <c r="D48" s="27"/>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="27"/>
-      <c r="B49" s="27"/>
-      <c r="C49" s="27"/>
-      <c r="D49" s="27"/>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="27"/>
-      <c r="B50" s="27"/>
-      <c r="C50" s="27"/>
-      <c r="D50" s="27"/>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="27"/>
-      <c r="B51" s="27"/>
-      <c r="C51" s="27"/>
-      <c r="D51" s="27"/>
+      <c r="B48" s="28"/>
+      <c r="C48" s="28"/>
+      <c r="D48" s="28"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="28"/>
+      <c r="B49" s="28"/>
+      <c r="C49" s="28"/>
+      <c r="D49" s="28"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="28"/>
+      <c r="B50" s="28"/>
+      <c r="C50" s="28"/>
+      <c r="D50" s="28"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="28"/>
+      <c r="B51" s="28"/>
+      <c r="C51" s="28"/>
+      <c r="D51" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1455,97 +1459,97 @@
   <dimension ref="A1:C12"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="44"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="28" t="s">
+    <row r="2" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="29" t="s">
         <v>71</v>
       </c>
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="29" t="s">
         <v>72</v>
       </c>
-      <c r="C2" s="28" t="s">
+      <c r="C2" s="29" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="29" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="30" t="s">
         <v>74</v>
       </c>
-      <c r="B3" s="30" t="n">
+      <c r="B3" s="31" t="n">
         <v>0.015</v>
       </c>
-      <c r="C3" s="29" t="s">
+      <c r="C3" s="30" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="29" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="30" t="n">
+      <c r="B4" s="31" t="n">
         <v>0.03</v>
       </c>
-      <c r="C4" s="29" t="s">
+      <c r="C4" s="30" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="29" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="30" t="s">
         <v>77</v>
       </c>
-      <c r="B5" s="30" t="n">
+      <c r="B5" s="31" t="n">
         <v>0.045</v>
       </c>
-      <c r="C5" s="29" t="s">
+      <c r="C5" s="30" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="29" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="30" t="s">
         <v>79</v>
       </c>
-      <c r="B6" s="30" t="n">
-        <v>0.029</v>
-      </c>
-      <c r="C6" s="29" t="s">
+      <c r="B6" s="31" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="C6" s="30" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="27" t="s">
+      <c r="A8" s="28" t="s">
         <v>81</v>
       </c>
-      <c r="B8" s="27"/>
-      <c r="C8" s="27"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="27"/>
-      <c r="B9" s="27"/>
-      <c r="C9" s="27"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="27"/>
-      <c r="B10" s="27"/>
-      <c r="C10" s="27"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="27"/>
-      <c r="B11" s="27"/>
-      <c r="C11" s="27"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="27"/>
-      <c r="B12" s="27"/>
-      <c r="C12" s="27"/>
+      <c r="B8" s="28"/>
+      <c r="C8" s="28"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="28"/>
+      <c r="B9" s="28"/>
+      <c r="C9" s="28"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="28"/>
+      <c r="B10" s="28"/>
+      <c r="C10" s="28"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="28"/>
+      <c r="B11" s="28"/>
+      <c r="C11" s="28"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="28"/>
+      <c r="B12" s="28"/>
+      <c r="C12" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1569,350 +1573,350 @@
   <dimension ref="A1:J15"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="17"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="31" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B4" s="32" t="s">
         <v>38</v>
       </c>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="31"/>
-      <c r="F4" s="31" t="s">
+      <c r="C4" s="32"/>
+      <c r="D4" s="32"/>
+      <c r="E4" s="32"/>
+      <c r="F4" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="G4" s="31"/>
-      <c r="H4" s="31"/>
-      <c r="I4" s="31"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="32" t="s">
+      <c r="G4" s="32"/>
+      <c r="H4" s="32"/>
+      <c r="I4" s="32"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="32" t="s">
+      <c r="B5" s="33" t="s">
         <v>84</v>
       </c>
-      <c r="C5" s="32" t="s">
+      <c r="C5" s="33" t="s">
         <v>85</v>
       </c>
-      <c r="D5" s="32" t="s">
+      <c r="D5" s="33" t="s">
         <v>86</v>
       </c>
-      <c r="E5" s="32" t="s">
+      <c r="E5" s="33" t="s">
         <v>87</v>
       </c>
-      <c r="F5" s="32" t="s">
+      <c r="F5" s="33" t="s">
         <v>84</v>
       </c>
-      <c r="G5" s="32" t="s">
+      <c r="G5" s="33" t="s">
         <v>85</v>
       </c>
-      <c r="H5" s="32" t="s">
+      <c r="H5" s="33" t="s">
         <v>86</v>
       </c>
-      <c r="I5" s="32" t="s">
+      <c r="I5" s="33" t="s">
         <v>87</v>
       </c>
-      <c r="J5" s="32" t="s">
+      <c r="J5" s="33" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="33" t="n">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="34" t="n">
         <v>1000</v>
       </c>
-      <c r="B6" s="34" t="n">
+      <c r="B6" s="35" t="n">
         <f aca="false">(IF(Estimator!$B$28&gt;0,MIN(Estimator!$B$8,ROUNDDOWN($A6/Estimator!$B$28,0)),0))*Estimator!$B$28</f>
         <v>999.979854</v>
       </c>
-      <c r="C6" s="35" t="n">
+      <c r="C6" s="36" t="n">
         <f aca="false">(IF(Estimator!$B$28&gt;0,MIN(Estimator!$B$8,ROUNDDOWN($A6/Estimator!$B$28,0)),0))*Estimator!$B$19*Estimator!$B$21</f>
         <v>29.36103</v>
       </c>
-      <c r="D6" s="36" t="n">
+      <c r="D6" s="37" t="n">
         <f aca="false">IF(C6&gt;0,B6/C6,"n/a")</f>
         <v>34.058064516129</v>
       </c>
-      <c r="E6" s="37" t="n">
+      <c r="E6" s="38" t="n">
         <f aca="false">IF(B6&gt;0,(C6*Estimator!$B$43-B6)/B6,0)</f>
         <v>0.468081075961357</v>
       </c>
-      <c r="F6" s="34" t="n">
+      <c r="F6" s="35" t="n">
         <f aca="false">(IF(Estimator!$C$28&gt;0,MIN(Estimator!$B$8,ROUNDDOWN($A6/Estimator!$C$28,0)),0))*Estimator!$C$28</f>
         <v>999.983964</v>
       </c>
-      <c r="G6" s="35" t="n">
+      <c r="G6" s="36" t="n">
         <f aca="false">(IF(Estimator!$C$28&gt;0,MIN(Estimator!$B$8,ROUNDDOWN($A6/Estimator!$C$28,0)),0))*Estimator!$C$19*Estimator!$C$21</f>
         <v>137.6333</v>
       </c>
-      <c r="H6" s="36" t="n">
+      <c r="H6" s="37" t="n">
         <f aca="false">IF(G6&gt;0,F6/G6,"n/a")</f>
         <v>7.26556701030928</v>
       </c>
-      <c r="I6" s="37" t="n">
+      <c r="I6" s="38" t="n">
         <f aca="false">IF(F6&gt;0,(G6*Estimator!$C$43-F6)/F6,0)</f>
         <v>13.4517282479142</v>
       </c>
-      <c r="J6" s="38" t="str">
+      <c r="J6" s="39" t="str">
         <f aca="false">IF(E6&gt;=Estimator!$B$7,"MEETS TARGET","BELOW TARGET")</f>
         <v>BELOW TARGET</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="33" t="n">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="34" t="n">
         <v>2500</v>
       </c>
-      <c r="B7" s="34" t="n">
+      <c r="B7" s="35" t="n">
         <f aca="false">(IF(Estimator!$B$28&gt;0,MIN(Estimator!$B$8,ROUNDDOWN($A7/Estimator!$B$28,0)),0))*Estimator!$B$28</f>
         <v>2499.997146</v>
       </c>
-      <c r="C7" s="35" t="n">
+      <c r="C7" s="36" t="n">
         <f aca="false">(IF(Estimator!$B$28&gt;0,MIN(Estimator!$B$8,ROUNDDOWN($A7/Estimator!$B$28,0)),0))*Estimator!$B$19*Estimator!$B$21</f>
         <v>73.40397</v>
       </c>
-      <c r="D7" s="36" t="n">
+      <c r="D7" s="37" t="n">
         <f aca="false">IF(C7&gt;0,B7/C7,"n/a")</f>
         <v>34.058064516129</v>
       </c>
-      <c r="E7" s="37" t="n">
+      <c r="E7" s="38" t="n">
         <f aca="false">IF(B7&gt;0,(C7*Estimator!$B$43-B7)/B7,0)</f>
         <v>0.468081075961356</v>
       </c>
-      <c r="F7" s="34" t="n">
+      <c r="F7" s="35" t="n">
         <f aca="false">(IF(Estimator!$C$28&gt;0,MIN(Estimator!$B$8,ROUNDDOWN($A7/Estimator!$C$28,0)),0))*Estimator!$C$28</f>
         <v>2499.995148</v>
       </c>
-      <c r="G7" s="35" t="n">
+      <c r="G7" s="36" t="n">
         <f aca="false">(IF(Estimator!$C$28&gt;0,MIN(Estimator!$B$8,ROUNDDOWN($A7/Estimator!$C$28,0)),0))*Estimator!$C$19*Estimator!$C$21</f>
         <v>344.0881</v>
       </c>
-      <c r="H7" s="36" t="n">
+      <c r="H7" s="37" t="n">
         <f aca="false">IF(G7&gt;0,F7/G7,"n/a")</f>
         <v>7.26556701030928</v>
       </c>
-      <c r="I7" s="37" t="n">
+      <c r="I7" s="38" t="n">
         <f aca="false">IF(F7&gt;0,(G7*Estimator!$C$43-F7)/F7,0)</f>
         <v>13.4517282479142</v>
       </c>
-      <c r="J7" s="38" t="str">
+      <c r="J7" s="39" t="str">
         <f aca="false">IF(E7&gt;=Estimator!$B$7,"MEETS TARGET","BELOW TARGET")</f>
         <v>BELOW TARGET</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="33" t="n">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="34" t="n">
         <v>5000</v>
       </c>
-      <c r="B8" s="34" t="n">
+      <c r="B8" s="35" t="n">
         <f aca="false">(IF(Estimator!$B$28&gt;0,MIN(Estimator!$B$8,ROUNDDOWN($A8/Estimator!$B$28,0)),0))*Estimator!$B$28</f>
         <v>3167.4</v>
       </c>
-      <c r="C8" s="35" t="n">
+      <c r="C8" s="36" t="n">
         <f aca="false">(IF(Estimator!$B$28&gt;0,MIN(Estimator!$B$8,ROUNDDOWN($A8/Estimator!$B$28,0)),0))*Estimator!$B$19*Estimator!$B$21</f>
         <v>93</v>
       </c>
-      <c r="D8" s="36" t="n">
+      <c r="D8" s="37" t="n">
         <f aca="false">IF(C8&gt;0,B8/C8,"n/a")</f>
         <v>34.058064516129</v>
       </c>
-      <c r="E8" s="37" t="n">
+      <c r="E8" s="38" t="n">
         <f aca="false">IF(B8&gt;0,(C8*Estimator!$B$43-B8)/B8,0)</f>
         <v>0.468081075961356</v>
       </c>
-      <c r="F8" s="34" t="n">
+      <c r="F8" s="35" t="n">
         <f aca="false">(IF(Estimator!$C$28&gt;0,MIN(Estimator!$B$8,ROUNDDOWN($A8/Estimator!$C$28,0)),0))*Estimator!$C$28</f>
         <v>3523.8</v>
       </c>
-      <c r="G8" s="35" t="n">
+      <c r="G8" s="36" t="n">
         <f aca="false">(IF(Estimator!$C$28&gt;0,MIN(Estimator!$B$8,ROUNDDOWN($A8/Estimator!$C$28,0)),0))*Estimator!$C$19*Estimator!$C$21</f>
         <v>485</v>
       </c>
-      <c r="H8" s="36" t="n">
+      <c r="H8" s="37" t="n">
         <f aca="false">IF(G8&gt;0,F8/G8,"n/a")</f>
         <v>7.26556701030928</v>
       </c>
-      <c r="I8" s="37" t="n">
+      <c r="I8" s="38" t="n">
         <f aca="false">IF(F8&gt;0,(G8*Estimator!$C$43-F8)/F8,0)</f>
         <v>13.4517282479142</v>
       </c>
-      <c r="J8" s="38" t="str">
+      <c r="J8" s="39" t="str">
         <f aca="false">IF(E8&gt;=Estimator!$B$7,"MEETS TARGET","BELOW TARGET")</f>
         <v>BELOW TARGET</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="33" t="n">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="34" t="n">
         <v>10000</v>
       </c>
-      <c r="B9" s="34" t="n">
+      <c r="B9" s="35" t="n">
         <f aca="false">(IF(Estimator!$B$28&gt;0,MIN(Estimator!$B$8,ROUNDDOWN($A9/Estimator!$B$28,0)),0))*Estimator!$B$28</f>
         <v>3167.4</v>
       </c>
-      <c r="C9" s="35" t="n">
+      <c r="C9" s="36" t="n">
         <f aca="false">(IF(Estimator!$B$28&gt;0,MIN(Estimator!$B$8,ROUNDDOWN($A9/Estimator!$B$28,0)),0))*Estimator!$B$19*Estimator!$B$21</f>
         <v>93</v>
       </c>
-      <c r="D9" s="36" t="n">
+      <c r="D9" s="37" t="n">
         <f aca="false">IF(C9&gt;0,B9/C9,"n/a")</f>
         <v>34.058064516129</v>
       </c>
-      <c r="E9" s="37" t="n">
+      <c r="E9" s="38" t="n">
         <f aca="false">IF(B9&gt;0,(C9*Estimator!$B$43-B9)/B9,0)</f>
         <v>0.468081075961356</v>
       </c>
-      <c r="F9" s="34" t="n">
+      <c r="F9" s="35" t="n">
         <f aca="false">(IF(Estimator!$C$28&gt;0,MIN(Estimator!$B$8,ROUNDDOWN($A9/Estimator!$C$28,0)),0))*Estimator!$C$28</f>
         <v>3523.8</v>
       </c>
-      <c r="G9" s="35" t="n">
+      <c r="G9" s="36" t="n">
         <f aca="false">(IF(Estimator!$C$28&gt;0,MIN(Estimator!$B$8,ROUNDDOWN($A9/Estimator!$C$28,0)),0))*Estimator!$C$19*Estimator!$C$21</f>
         <v>485</v>
       </c>
-      <c r="H9" s="36" t="n">
+      <c r="H9" s="37" t="n">
         <f aca="false">IF(G9&gt;0,F9/G9,"n/a")</f>
         <v>7.26556701030928</v>
       </c>
-      <c r="I9" s="37" t="n">
+      <c r="I9" s="38" t="n">
         <f aca="false">IF(F9&gt;0,(G9*Estimator!$C$43-F9)/F9,0)</f>
         <v>13.4517282479142</v>
       </c>
-      <c r="J9" s="38" t="str">
+      <c r="J9" s="39" t="str">
         <f aca="false">IF(E9&gt;=Estimator!$B$7,"MEETS TARGET","BELOW TARGET")</f>
         <v>BELOW TARGET</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="33" t="n">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="34" t="n">
         <v>25000</v>
       </c>
-      <c r="B10" s="34" t="n">
+      <c r="B10" s="35" t="n">
         <f aca="false">(IF(Estimator!$B$28&gt;0,MIN(Estimator!$B$8,ROUNDDOWN($A10/Estimator!$B$28,0)),0))*Estimator!$B$28</f>
         <v>3167.4</v>
       </c>
-      <c r="C10" s="35" t="n">
+      <c r="C10" s="36" t="n">
         <f aca="false">(IF(Estimator!$B$28&gt;0,MIN(Estimator!$B$8,ROUNDDOWN($A10/Estimator!$B$28,0)),0))*Estimator!$B$19*Estimator!$B$21</f>
         <v>93</v>
       </c>
-      <c r="D10" s="36" t="n">
+      <c r="D10" s="37" t="n">
         <f aca="false">IF(C10&gt;0,B10/C10,"n/a")</f>
         <v>34.058064516129</v>
       </c>
-      <c r="E10" s="37" t="n">
+      <c r="E10" s="38" t="n">
         <f aca="false">IF(B10&gt;0,(C10*Estimator!$B$43-B10)/B10,0)</f>
         <v>0.468081075961356</v>
       </c>
-      <c r="F10" s="34" t="n">
+      <c r="F10" s="35" t="n">
         <f aca="false">(IF(Estimator!$C$28&gt;0,MIN(Estimator!$B$8,ROUNDDOWN($A10/Estimator!$C$28,0)),0))*Estimator!$C$28</f>
         <v>3523.8</v>
       </c>
-      <c r="G10" s="35" t="n">
+      <c r="G10" s="36" t="n">
         <f aca="false">(IF(Estimator!$C$28&gt;0,MIN(Estimator!$B$8,ROUNDDOWN($A10/Estimator!$C$28,0)),0))*Estimator!$C$19*Estimator!$C$21</f>
         <v>485</v>
       </c>
-      <c r="H10" s="36" t="n">
+      <c r="H10" s="37" t="n">
         <f aca="false">IF(G10&gt;0,F10/G10,"n/a")</f>
         <v>7.26556701030928</v>
       </c>
-      <c r="I10" s="37" t="n">
+      <c r="I10" s="38" t="n">
         <f aca="false">IF(F10&gt;0,(G10*Estimator!$C$43-F10)/F10,0)</f>
         <v>13.4517282479142</v>
       </c>
-      <c r="J10" s="38" t="str">
+      <c r="J10" s="39" t="str">
         <f aca="false">IF(E10&gt;=Estimator!$B$7,"MEETS TARGET","BELOW TARGET")</f>
         <v>BELOW TARGET</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="33" t="n">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="34" t="n">
         <v>50000</v>
       </c>
-      <c r="B11" s="34" t="n">
+      <c r="B11" s="35" t="n">
         <f aca="false">(IF(Estimator!$B$28&gt;0,MIN(Estimator!$B$8,ROUNDDOWN($A11/Estimator!$B$28,0)),0))*Estimator!$B$28</f>
         <v>3167.4</v>
       </c>
-      <c r="C11" s="35" t="n">
+      <c r="C11" s="36" t="n">
         <f aca="false">(IF(Estimator!$B$28&gt;0,MIN(Estimator!$B$8,ROUNDDOWN($A11/Estimator!$B$28,0)),0))*Estimator!$B$19*Estimator!$B$21</f>
         <v>93</v>
       </c>
-      <c r="D11" s="36" t="n">
+      <c r="D11" s="37" t="n">
         <f aca="false">IF(C11&gt;0,B11/C11,"n/a")</f>
         <v>34.058064516129</v>
       </c>
-      <c r="E11" s="37" t="n">
+      <c r="E11" s="38" t="n">
         <f aca="false">IF(B11&gt;0,(C11*Estimator!$B$43-B11)/B11,0)</f>
         <v>0.468081075961356</v>
       </c>
-      <c r="F11" s="34" t="n">
+      <c r="F11" s="35" t="n">
         <f aca="false">(IF(Estimator!$C$28&gt;0,MIN(Estimator!$B$8,ROUNDDOWN($A11/Estimator!$C$28,0)),0))*Estimator!$C$28</f>
         <v>3523.8</v>
       </c>
-      <c r="G11" s="35" t="n">
+      <c r="G11" s="36" t="n">
         <f aca="false">(IF(Estimator!$C$28&gt;0,MIN(Estimator!$B$8,ROUNDDOWN($A11/Estimator!$C$28,0)),0))*Estimator!$C$19*Estimator!$C$21</f>
         <v>485</v>
       </c>
-      <c r="H11" s="36" t="n">
+      <c r="H11" s="37" t="n">
         <f aca="false">IF(G11&gt;0,F11/G11,"n/a")</f>
         <v>7.26556701030928</v>
       </c>
-      <c r="I11" s="37" t="n">
+      <c r="I11" s="38" t="n">
         <f aca="false">IF(F11&gt;0,(G11*Estimator!$C$43-F11)/F11,0)</f>
         <v>13.4517282479142</v>
       </c>
-      <c r="J11" s="38" t="str">
+      <c r="J11" s="39" t="str">
         <f aca="false">IF(E11&gt;=Estimator!$B$7,"MEETS TARGET","BELOW TARGET")</f>
         <v>BELOW TARGET</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="27" t="s">
+      <c r="A13" s="28" t="s">
         <v>89</v>
       </c>
-      <c r="B13" s="27"/>
-      <c r="C13" s="27"/>
-      <c r="D13" s="27"/>
-      <c r="E13" s="27"/>
-      <c r="F13" s="27"/>
-      <c r="G13" s="27"/>
-      <c r="H13" s="27"/>
-      <c r="I13" s="27"/>
-      <c r="J13" s="27"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="27"/>
-      <c r="B14" s="27"/>
-      <c r="C14" s="27"/>
-      <c r="D14" s="27"/>
-      <c r="E14" s="27"/>
-      <c r="F14" s="27"/>
-      <c r="G14" s="27"/>
-      <c r="H14" s="27"/>
-      <c r="I14" s="27"/>
-      <c r="J14" s="27"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="27"/>
-      <c r="B15" s="27"/>
-      <c r="C15" s="27"/>
-      <c r="D15" s="27"/>
-      <c r="E15" s="27"/>
-      <c r="F15" s="27"/>
-      <c r="G15" s="27"/>
-      <c r="H15" s="27"/>
-      <c r="I15" s="27"/>
-      <c r="J15" s="27"/>
+      <c r="B13" s="28"/>
+      <c r="C13" s="28"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="28"/>
+      <c r="F13" s="28"/>
+      <c r="G13" s="28"/>
+      <c r="H13" s="28"/>
+      <c r="I13" s="28"/>
+      <c r="J13" s="28"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="28"/>
+      <c r="B14" s="28"/>
+      <c r="C14" s="28"/>
+      <c r="D14" s="28"/>
+      <c r="E14" s="28"/>
+      <c r="F14" s="28"/>
+      <c r="G14" s="28"/>
+      <c r="H14" s="28"/>
+      <c r="I14" s="28"/>
+      <c r="J14" s="28"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="28"/>
+      <c r="B15" s="28"/>
+      <c r="C15" s="28"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="28"/>
+      <c r="F15" s="28"/>
+      <c r="G15" s="28"/>
+      <c r="H15" s="28"/>
+      <c r="I15" s="28"/>
+      <c r="J15" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>